<commit_message>
Backfill spreadsheet rows for batch 2 (Blackrock, Paradromics, Soterix, Cala, Saluda)
Another session already fixed the BACKLOG/tech-tree/changelog gaps for this
batch; this adds the one piece still missing — the Master sheet and
category-sheet rows in data/neuromodulation_startups.xlsx.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0141ut2GnnMPpbzHjZKr1k1F
</commit_message>
<xml_diff>
--- a/data/neuromodulation_startups.xlsx
+++ b/data/neuromodulation_startups.xlsx
@@ -666,7 +666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1834,6 +1834,366 @@
       <c r="N16" s="9" t="inlineStr">
         <is>
           <t>docs/profiles/neuro-musculoskeletal-pain-movement/onward-medical.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Blackrock Neurotech</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Cognitive Disorders / Neural Interface</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Salt Lake City, Utah, USA</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2006</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Private; funding not publicly disclosed. Decades-long BrainGate consortium partner.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Primary motor cortex (M1), penetrating 96-128 channel Utah Array via craniotomy; single-unit action-potential recording.</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Motor cortex population-vector coding of intended movement remains intact after paralysis (Georgopoulos et al. 1986, Science); decoders map spike trains to movement intent.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>~5.5M Americans with paralysis, ~200k+ US ALS; ~1-2M globally with severe paralysis addressable for intracortical BCI. Market ~$50-100M today, projected $6-10B by 2030-35 if adoption accelerates.</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Utah Array (96/128-channel penetrating microelectrode grid) + amplifiers/ADC + percutaneous or wireless telemetry; proprietary decoding software drives cursor/robotic-arm/prosthetic control.</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Longest human-implant track record (BrainGate, since 2004) of any intracortical BCI; FDA-familiar via multiple IDE trials; vs. Paradromics' much higher (10,000+) channel count still in preclinical/early trial stage.</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Craniotomy risk (~0.5-1% mortality, 1-2% infection); $100k-200k device+surgery cost, rarely reimbursed; weekly recalibration and daily training burden; only ~5-10 US centers can implant/support.</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Recording quality degrades 6-24mo post-implant (glial scarring); long-term (&gt;2yr) human data sparse; no CPT reimbursement codes yet; FDA pathway (De Novo/PMA) for intracortical BCI still undefined.</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>No full FDA approval yet (as of Sept 2026); operating under IDE via BrainGate consortium (Brown, Stanford, Mass General). Published &gt;95% cursor-task accuracy, 1-3 bits/sec information transfer. Projected first De Novo approval 2027-2030.</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>docs/profiles/cognitive-disorders-neural-interface/blackrock-neurotech.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Paradromics, Inc.</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Cognitive Disorders / Neural Interface</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Austin, Texas, USA</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Private. $20M+ Series A (2021); Series B in progress (2025).</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Primary motor + somatosensory cortex (M1/S1), penetrating ultra-high-channel-count (10,000+) 'hyperdimensional electrode' array; bidirectional recording + stimulation.</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Same population-vector motor coding as other intracortical BCIs, but 100x more channels enables richer/redundant decoding; S1 stimulation can evoke artificial tactile percepts for closed-loop sensorimotor feedback.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Same addressable paralysis/ALS population as Blackrock (~1-2M severe cases globally). Intracortical BCI market ~$50-100M now; Paradromics potential TAM $1-5B if high-channel systems reach approval.</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>10,000+ microscale penetrating electrodes with on-implant analog processing/multiplexing, wireless telemetry, GPU-based real-time decoding, bidirectional motor+sensory closed-loop software.</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>100x the channel count of Blackrock's Utah Array; only bidirectional (motor decode + sensory feedback) system in this cohort; trade-off is higher surgical complexity/cost and far less clinical data than Blackrock.</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Estimated $200k-500k device+surgery cost; 6-8+ hour surgery requiring highly specialized neurosurgeons; only 1-2 centers currently; unproven long-term durability of 10,000-electrode arrays.</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>No precedent for FDA review of a 10,000-channel implant; 'curse of dimensionality' risk that more channels don't proportionally improve decoding; bidirectional sensory feedback human experience limited to 1-2 published cases.</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Preclinical/early feasibility stage; IND/IDE engagement pending as of 2026. Early feasibility study (n=4-8) recruiting 2024-2026; first human implant trial expected 2026-2027, FDA approval not expected before 2028-2030.</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>docs/profiles/cognitive-disorders-neural-interface/paradromics.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Soterix Medical, Inc.</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Mental Health / Psychiatric</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>New York, New York, USA</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Private. $20M+ raised; exact amounts not publicly disclosed.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Dorsolateral prefrontal cortex (DLPFC), left hemisphere anode; transcranial direct current stimulation (tDCS/HDtDCS) via scalp electrodes, 1-2mA for 20-40min.</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>MDD linked to left DLPFC hypoactivity; weak anodal tDCS current is hypothesized to increase cortical excitability in the underlying region, partially normalizing this asymmetry.</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Global depression treatment market $15-20B annually (drugs+psychotherapy+devices). tDCS device market ~$50-100M today, projected $300M-1B by 2030; Soterix estimated 5-15% share if approved.</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Conventional 2-electrode tDCS and High-Definition tDCS (smaller electrodes, more focal current) devices; clinician- or protocol-administered scalp stimulation sessions.</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>One of the longest-established tDCS device makers (research + clinical); HDtDCS offers more focal targeting than conventional 2-electrode tDCS or competitors like Flow Neuroscience's at-home device.</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>No FDA approval yet for depression as of Sept 2026 (research-use-only 510(k) clearance); requires clinician administration/facility visits for clinical protocols; efficacy vs. sham still debated in the tDCS literature.</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>tDCS mechanism (weak, diffuse subthreshold current) has a less mature efficacy evidence base than TMS; De Novo/PMA pathway for a clinical depression claim not yet cleared.</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>No formal FDA clinical-treatment approval for depression as of Sept 2026; devices cleared 510(k) for research use only; pursuing De Novo/PMA with RCT data, decision expected 2027-2028.</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>docs/profiles/mental-health-psychiatric/soterix-medical.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Cala Health</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Neuro-Musculoskeletal / Pain / Movement</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>San Francisco, California, USA</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Private. $45M Series A (2019); Series B amount not publicly disclosed.</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Radial and median/ulnar nerves at the wrist; non-invasive wearable (Cala Trio) delivers transcutaneous high-frequency nerve stimulation via adhesive electrodes.</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Peripheral afferent stimulation is hypothesized to disrupt the central tremor oscillator circuit (cerebello-thalamo-cortical loop) implicated in essential tremor, reducing tremor amplitude for a period after stimulation.</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Essential tremor device/treatment market ~$200-500M annually; non-invasive tremor neuromodulation segment projected $100M-1B by 2030. Cala Trio priced ~$3k-5k per device.</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Wrist-worn stimulator (Cala Trio) with adhesive forearm/wrist electrodes; patient self-administers on-demand or scheduled stimulation sessions at home, no implant required.</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Fully non-invasive, patient-administered, no surgery required — contrasts with DBS or implanted peripheral stimulators for tremor; wearable form factor targets patients unwilling/ineligible for surgical options.</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Effect is often transient (hours, not permanent); requires repeated daily sessions; out-of-pocket cost and limited insurance coverage; efficacy varies by patient/tremor severity.</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Preclinical/early-clinical stage per company disclosures; De Novo pathway likely; FDA clearance timeline projected 2027-2029 pending trial progress.</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>No PMA/De Novo clearance confirmed as of profile date; IND/FDA discussions ongoing. (Note: commercial device has FDA clearance in the broader market — verify current regulatory status before investment decisions.)</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>docs/profiles/neuro-musculoskeletal-pain-movement/cala-health.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Saluda Medical, Inc.</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Neuro-Musculoskeletal / Pain / Movement</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Sydney, Australia (HQ); Boston, MA, USA (US ops)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Private. $100M+ Series B (2018); backed by venture and strategic investors.</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Dorsal root ganglia (DRG) / dorsal column spinal cord; implantable epidural lead delivers electrical stimulation with real-time evoked compound action potential (ECAP) feedback for closed-loop dose control.</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Gate control theory (Melzack &amp; Wall 1965): stimulating large-diameter dorsal column fibers inhibits nociceptive transmission. ECAP recording lets the device measure the neural response to each pulse and auto-adjust amplitude, unlike fixed-output SCS.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Global SCS market ~$3-4B annually (2024); closed-loop SCS segment projected $500M-2B by 2030. Saluda estimated 5-15% share if regulatory/reimbursement succeed.</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Percutaneous epidural lead + implantable pulse generator; Evoke System measures ECAPs after each stimulus and closed-loop adjusts stimulation amplitude to keep neural activation within a target therapeutic window.</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Only commercial SCS system with objective, real-time neural-response (ECAP) feedback vs. fixed-output competitors (Medtronic, Boston Scientific, Abbott, Nevro); aims to reduce both under- and over-stimulation.</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Same implant risks as any SCS (lead migration, infection, surgical revision); requires trial period before permanent implant; premium pricing vs. conventional SCS.</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Closed-loop advantage is well-differentiated on paper but long-term comparative-effectiveness data vs. fixed-output competitors is still accumulating.</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Traditional SCS competitors approved via 510(k); Saluda pursuing breakthrough designation / 510(k) or De Novo for closed-loop claim, FDA clearance expected 2026-2027 per profile. (Note: Evoke has received FDA approval in the broader market — verify current regulatory status before investment decisions.)</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>docs/profiles/neuro-musculoskeletal-pain-movement/saluda-medical.md</t>
         </is>
       </c>
     </row>
@@ -2166,7 +2526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2545,6 +2905,150 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Blackrock Neurotech</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Cognitive Disorders / Neural Interface</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Salt Lake City, Utah, USA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2006</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Private; funding not publicly disclosed. Decades-long BrainGate consortium partner.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Primary motor cortex (M1), penetrating 96-128 channel Utah Array via craniotomy; single-unit action-potential recording.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Motor cortex population-vector coding of intended movement remains intact after paralysis (Georgopoulos et al. 1986, Science); decoders map spike trains to movement intent.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>~5.5M Americans with paralysis, ~200k+ US ALS; ~1-2M globally with severe paralysis addressable for intracortical BCI. Market ~$50-100M today, projected $6-10B by 2030-35 if adoption accelerates.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Utah Array (96/128-channel penetrating microelectrode grid) + amplifiers/ADC + percutaneous or wireless telemetry; proprietary decoding software drives cursor/robotic-arm/prosthetic control.</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Longest human-implant track record (BrainGate, since 2004) of any intracortical BCI; FDA-familiar via multiple IDE trials; vs. Paradromics' much higher (10,000+) channel count still in preclinical/early trial stage.</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Craniotomy risk (~0.5-1% mortality, 1-2% infection); $100k-200k device+surgery cost, rarely reimbursed; weekly recalibration and daily training burden; only ~5-10 US centers can implant/support.</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Recording quality degrades 6-24mo post-implant (glial scarring); long-term (&gt;2yr) human data sparse; no CPT reimbursement codes yet; FDA pathway (De Novo/PMA) for intracortical BCI still undefined.</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>No full FDA approval yet (as of Sept 2026); operating under IDE via BrainGate consortium (Brown, Stanford, Mass General). Published &gt;95% cursor-task accuracy, 1-3 bits/sec information transfer. Projected first De Novo approval 2027-2030.</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>docs/profiles/cognitive-disorders-neural-interface/blackrock-neurotech.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Paradromics, Inc.</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Cognitive Disorders / Neural Interface</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Austin, Texas, USA</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Private. $20M+ Series A (2021); Series B in progress (2025).</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Primary motor + somatosensory cortex (M1/S1), penetrating ultra-high-channel-count (10,000+) 'hyperdimensional electrode' array; bidirectional recording + stimulation.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Same population-vector motor coding as other intracortical BCIs, but 100x more channels enables richer/redundant decoding; S1 stimulation can evoke artificial tactile percepts for closed-loop sensorimotor feedback.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Same addressable paralysis/ALS population as Blackrock (~1-2M severe cases globally). Intracortical BCI market ~$50-100M now; Paradromics potential TAM $1-5B if high-channel systems reach approval.</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>10,000+ microscale penetrating electrodes with on-implant analog processing/multiplexing, wireless telemetry, GPU-based real-time decoding, bidirectional motor+sensory closed-loop software.</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>100x the channel count of Blackrock's Utah Array; only bidirectional (motor decode + sensory feedback) system in this cohort; trade-off is higher surgical complexity/cost and far less clinical data than Blackrock.</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Estimated $200k-500k device+surgery cost; 6-8+ hour surgery requiring highly specialized neurosurgeons; only 1-2 centers currently; unproven long-term durability of 10,000-electrode arrays.</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>No precedent for FDA review of a 10,000-channel implant; 'curse of dimensionality' risk that more channels don't proportionally improve decoding; bidirectional sensory feedback human experience limited to 1-2 published cases.</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Preclinical/early feasibility stage; IND/IDE engagement pending as of 2026. Early feasibility study (n=4-8) recruiting 2024-2026; first human implant trial expected 2026-2027, FDA approval not expected before 2028-2030.</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>docs/profiles/cognitive-disorders-neural-interface/paradromics.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2556,7 +3060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2935,6 +3439,78 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Soterix Medical, Inc.</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mental Health / Psychiatric</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>New York, New York, USA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Private. $20M+ raised; exact amounts not publicly disclosed.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Dorsolateral prefrontal cortex (DLPFC), left hemisphere anode; transcranial direct current stimulation (tDCS/HDtDCS) via scalp electrodes, 1-2mA for 20-40min.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>MDD linked to left DLPFC hypoactivity; weak anodal tDCS current is hypothesized to increase cortical excitability in the underlying region, partially normalizing this asymmetry.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Global depression treatment market $15-20B annually (drugs+psychotherapy+devices). tDCS device market ~$50-100M today, projected $300M-1B by 2030; Soterix estimated 5-15% share if approved.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Conventional 2-electrode tDCS and High-Definition tDCS (smaller electrodes, more focal current) devices; clinician- or protocol-administered scalp stimulation sessions.</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>One of the longest-established tDCS device makers (research + clinical); HDtDCS offers more focal targeting than conventional 2-electrode tDCS or competitors like Flow Neuroscience's at-home device.</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>No FDA approval yet for depression as of Sept 2026 (research-use-only 510(k) clearance); requires clinician administration/facility visits for clinical protocols; efficacy vs. sham still debated in the tDCS literature.</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>tDCS mechanism (weak, diffuse subthreshold current) has a less mature efficacy evidence base than TMS; De Novo/PMA pathway for a clinical depression claim not yet cleared.</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>No formal FDA clinical-treatment approval for depression as of Sept 2026; devices cleared 510(k) for research use only; pursuing De Novo/PMA with RCT data, decision expected 2027-2028.</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>docs/profiles/mental-health-psychiatric/soterix-medical.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2946,7 +3522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3325,6 +3901,150 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Cala Health</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Neuro-Musculoskeletal / Pain / Movement</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>San Francisco, California, USA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Private. $45M Series A (2019); Series B amount not publicly disclosed.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Radial and median/ulnar nerves at the wrist; non-invasive wearable (Cala Trio) delivers transcutaneous high-frequency nerve stimulation via adhesive electrodes.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Peripheral afferent stimulation is hypothesized to disrupt the central tremor oscillator circuit (cerebello-thalamo-cortical loop) implicated in essential tremor, reducing tremor amplitude for a period after stimulation.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Essential tremor device/treatment market ~$200-500M annually; non-invasive tremor neuromodulation segment projected $100M-1B by 2030. Cala Trio priced ~$3k-5k per device.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Wrist-worn stimulator (Cala Trio) with adhesive forearm/wrist electrodes; patient self-administers on-demand or scheduled stimulation sessions at home, no implant required.</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Fully non-invasive, patient-administered, no surgery required — contrasts with DBS or implanted peripheral stimulators for tremor; wearable form factor targets patients unwilling/ineligible for surgical options.</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Effect is often transient (hours, not permanent); requires repeated daily sessions; out-of-pocket cost and limited insurance coverage; efficacy varies by patient/tremor severity.</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Preclinical/early-clinical stage per company disclosures; De Novo pathway likely; FDA clearance timeline projected 2027-2029 pending trial progress.</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>No PMA/De Novo clearance confirmed as of profile date; IND/FDA discussions ongoing. (Note: commercial device has FDA clearance in the broader market — verify current regulatory status before investment decisions.)</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>docs/profiles/neuro-musculoskeletal-pain-movement/cala-health.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Saluda Medical, Inc.</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Neuro-Musculoskeletal / Pain / Movement</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Sydney, Australia (HQ); Boston, MA, USA (US ops)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Private. $100M+ Series B (2018); backed by venture and strategic investors.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Dorsal root ganglia (DRG) / dorsal column spinal cord; implantable epidural lead delivers electrical stimulation with real-time evoked compound action potential (ECAP) feedback for closed-loop dose control.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Gate control theory (Melzack &amp; Wall 1965): stimulating large-diameter dorsal column fibers inhibits nociceptive transmission. ECAP recording lets the device measure the neural response to each pulse and auto-adjust amplitude, unlike fixed-output SCS.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Global SCS market ~$3-4B annually (2024); closed-loop SCS segment projected $500M-2B by 2030. Saluda estimated 5-15% share if regulatory/reimbursement succeed.</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Percutaneous epidural lead + implantable pulse generator; Evoke System measures ECAPs after each stimulus and closed-loop adjusts stimulation amplitude to keep neural activation within a target therapeutic window.</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Only commercial SCS system with objective, real-time neural-response (ECAP) feedback vs. fixed-output competitors (Medtronic, Boston Scientific, Abbott, Nevro); aims to reduce both under- and over-stimulation.</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Same implant risks as any SCS (lead migration, infection, surgical revision); requires trial period before permanent implant; premium pricing vs. conventional SCS.</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Closed-loop advantage is well-differentiated on paper but long-term comparative-effectiveness data vs. fixed-output competitors is still accumulating.</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Traditional SCS competitors approved via 510(k); Saluda pursuing breakthrough designation / 510(k) or De Novo for closed-loop claim, FDA clearance expected 2026-2027 per profile. (Note: Evoke has received FDA approval in the broader market — verify current regulatory status before investment decisions.)</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>docs/profiles/neuro-musculoskeletal-pain-movement/saluda-medical.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix spreadsheet formatting for batch 2 rows, add reusable update script
The Sept 13 backfill (7abdaf4) added 5 startup rows to
neuromodulation_startups.xlsx via raw openpyxl, which produced unstyled rows
(Calibri, no fill, no wrap, no border, no row height) instead of matching
the workbook's established per-category style.

- Fix formatting on all 10 affected rows (Master + 3 category sheets) to
  match the Arial/category-fill/wrap/border/130pt-row look of the original 15
- Add scripts/update_xlsx.py as the canonical way to add or fix spreadsheet
  rows; the daily research automation is now required to use it instead of
  ad-hoc openpyxl code, so this class of mistake can't recur
- Remove .DS_Store and a stray .patch file that a local auto-push watcher
  had swept into an earlier commit via a blind 'git add .'; add .gitignore

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012Rx7Ms9Dr8TYqWUVdNu1x1
</commit_message>
<xml_diff>
--- a/data/neuromodulation_startups.xlsx
+++ b/data/neuromodulation_startups.xlsx
@@ -102,7 +102,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -124,11 +124,17 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -156,6 +162,15 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1837,361 +1852,361 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="17" ht="130" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>Blackrock Neurotech</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>Cognitive Disorders / Neural Interface</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>Salt Lake City, Utah, USA</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="10" t="inlineStr">
         <is>
           <t>2006</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="10" t="inlineStr">
         <is>
           <t>Private; funding not publicly disclosed. Decades-long BrainGate consortium partner.</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="10" t="inlineStr">
         <is>
           <t>Primary motor cortex (M1), penetrating 96-128 channel Utah Array via craniotomy; single-unit action-potential recording.</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" s="10" t="inlineStr">
         <is>
           <t>Motor cortex population-vector coding of intended movement remains intact after paralysis (Georgopoulos et al. 1986, Science); decoders map spike trains to movement intent.</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H17" s="10" t="inlineStr">
         <is>
           <t>~5.5M Americans with paralysis, ~200k+ US ALS; ~1-2M globally with severe paralysis addressable for intracortical BCI. Market ~$50-100M today, projected $6-10B by 2030-35 if adoption accelerates.</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I17" s="10" t="inlineStr">
         <is>
           <t>Utah Array (96/128-channel penetrating microelectrode grid) + amplifiers/ADC + percutaneous or wireless telemetry; proprietary decoding software drives cursor/robotic-arm/prosthetic control.</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="J17" s="10" t="inlineStr">
         <is>
           <t>Longest human-implant track record (BrainGate, since 2004) of any intracortical BCI; FDA-familiar via multiple IDE trials; vs. Paradromics' much higher (10,000+) channel count still in preclinical/early trial stage.</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="K17" s="10" t="inlineStr">
         <is>
           <t>Craniotomy risk (~0.5-1% mortality, 1-2% infection); $100k-200k device+surgery cost, rarely reimbursed; weekly recalibration and daily training burden; only ~5-10 US centers can implant/support.</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="L17" s="10" t="inlineStr">
         <is>
           <t>Recording quality degrades 6-24mo post-implant (glial scarring); long-term (&gt;2yr) human data sparse; no CPT reimbursement codes yet; FDA pathway (De Novo/PMA) for intracortical BCI still undefined.</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="M17" s="10" t="inlineStr">
         <is>
           <t>No full FDA approval yet (as of Sept 2026); operating under IDE via BrainGate consortium (Brown, Stanford, Mass General). Published &gt;95% cursor-task accuracy, 1-3 bits/sec information transfer. Projected first De Novo approval 2027-2030.</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="N17" s="10" t="inlineStr">
         <is>
           <t>docs/profiles/cognitive-disorders-neural-interface/blackrock-neurotech.md</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="18" ht="130" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>Paradromics, Inc.</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>Cognitive Disorders / Neural Interface</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>Austin, Texas, USA</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>2015</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>Private. $20M+ Series A (2021); Series B in progress (2025).</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F18" s="10" t="inlineStr">
         <is>
           <t>Primary motor + somatosensory cortex (M1/S1), penetrating ultra-high-channel-count (10,000+) 'hyperdimensional electrode' array; bidirectional recording + stimulation.</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G18" s="10" t="inlineStr">
         <is>
           <t>Same population-vector motor coding as other intracortical BCIs, but 100x more channels enables richer/redundant decoding; S1 stimulation can evoke artificial tactile percepts for closed-loop sensorimotor feedback.</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="H18" s="10" t="inlineStr">
         <is>
           <t>Same addressable paralysis/ALS population as Blackrock (~1-2M severe cases globally). Intracortical BCI market ~$50-100M now; Paradromics potential TAM $1-5B if high-channel systems reach approval.</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="I18" s="10" t="inlineStr">
         <is>
           <t>10,000+ microscale penetrating electrodes with on-implant analog processing/multiplexing, wireless telemetry, GPU-based real-time decoding, bidirectional motor+sensory closed-loop software.</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="J18" s="10" t="inlineStr">
         <is>
           <t>100x the channel count of Blackrock's Utah Array; only bidirectional (motor decode + sensory feedback) system in this cohort; trade-off is higher surgical complexity/cost and far less clinical data than Blackrock.</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="K18" s="10" t="inlineStr">
         <is>
           <t>Estimated $200k-500k device+surgery cost; 6-8+ hour surgery requiring highly specialized neurosurgeons; only 1-2 centers currently; unproven long-term durability of 10,000-electrode arrays.</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="L18" s="10" t="inlineStr">
         <is>
           <t>No precedent for FDA review of a 10,000-channel implant; 'curse of dimensionality' risk that more channels don't proportionally improve decoding; bidirectional sensory feedback human experience limited to 1-2 published cases.</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="M18" s="10" t="inlineStr">
         <is>
           <t>Preclinical/early feasibility stage; IND/IDE engagement pending as of 2026. Early feasibility study (n=4-8) recruiting 2024-2026; first human implant trial expected 2026-2027, FDA approval not expected before 2028-2030.</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="N18" s="10" t="inlineStr">
         <is>
           <t>docs/profiles/cognitive-disorders-neural-interface/paradromics.md</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="19" ht="130" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>Soterix Medical, Inc.</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>Mental Health / Psychiatric</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>New York, New York, USA</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="11" t="inlineStr">
         <is>
           <t>2008</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="11" t="inlineStr">
         <is>
           <t>Private. $20M+ raised; exact amounts not publicly disclosed.</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F19" s="11" t="inlineStr">
         <is>
           <t>Dorsolateral prefrontal cortex (DLPFC), left hemisphere anode; transcranial direct current stimulation (tDCS/HDtDCS) via scalp electrodes, 1-2mA for 20-40min.</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G19" s="11" t="inlineStr">
         <is>
           <t>MDD linked to left DLPFC hypoactivity; weak anodal tDCS current is hypothesized to increase cortical excitability in the underlying region, partially normalizing this asymmetry.</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H19" s="11" t="inlineStr">
         <is>
           <t>Global depression treatment market $15-20B annually (drugs+psychotherapy+devices). tDCS device market ~$50-100M today, projected $300M-1B by 2030; Soterix estimated 5-15% share if approved.</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I19" s="11" t="inlineStr">
         <is>
           <t>Conventional 2-electrode tDCS and High-Definition tDCS (smaller electrodes, more focal current) devices; clinician- or protocol-administered scalp stimulation sessions.</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="J19" s="11" t="inlineStr">
         <is>
           <t>One of the longest-established tDCS device makers (research + clinical); HDtDCS offers more focal targeting than conventional 2-electrode tDCS or competitors like Flow Neuroscience's at-home device.</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="K19" s="11" t="inlineStr">
         <is>
           <t>No FDA approval yet for depression as of Sept 2026 (research-use-only 510(k) clearance); requires clinician administration/facility visits for clinical protocols; efficacy vs. sham still debated in the tDCS literature.</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="L19" s="11" t="inlineStr">
         <is>
           <t>tDCS mechanism (weak, diffuse subthreshold current) has a less mature efficacy evidence base than TMS; De Novo/PMA pathway for a clinical depression claim not yet cleared.</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="M19" s="11" t="inlineStr">
         <is>
           <t>No formal FDA clinical-treatment approval for depression as of Sept 2026; devices cleared 510(k) for research use only; pursuing De Novo/PMA with RCT data, decision expected 2027-2028.</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
+      <c r="N19" s="11" t="inlineStr">
         <is>
           <t>docs/profiles/mental-health-psychiatric/soterix-medical.md</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="20" ht="130" customHeight="1">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t>Cala Health</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>Neuro-Musculoskeletal / Pain / Movement</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="12" t="inlineStr">
         <is>
           <t>San Francisco, California, USA</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="12" t="inlineStr">
         <is>
           <t>2014</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="12" t="inlineStr">
         <is>
           <t>Private. $45M Series A (2019); Series B amount not publicly disclosed.</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F20" s="12" t="inlineStr">
         <is>
           <t>Radial and median/ulnar nerves at the wrist; non-invasive wearable (Cala Trio) delivers transcutaneous high-frequency nerve stimulation via adhesive electrodes.</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" s="12" t="inlineStr">
         <is>
           <t>Peripheral afferent stimulation is hypothesized to disrupt the central tremor oscillator circuit (cerebello-thalamo-cortical loop) implicated in essential tremor, reducing tremor amplitude for a period after stimulation.</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H20" s="12" t="inlineStr">
         <is>
           <t>Essential tremor device/treatment market ~$200-500M annually; non-invasive tremor neuromodulation segment projected $100M-1B by 2030. Cala Trio priced ~$3k-5k per device.</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I20" s="12" t="inlineStr">
         <is>
           <t>Wrist-worn stimulator (Cala Trio) with adhesive forearm/wrist electrodes; patient self-administers on-demand or scheduled stimulation sessions at home, no implant required.</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="J20" s="12" t="inlineStr">
         <is>
           <t>Fully non-invasive, patient-administered, no surgery required — contrasts with DBS or implanted peripheral stimulators for tremor; wearable form factor targets patients unwilling/ineligible for surgical options.</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="K20" s="12" t="inlineStr">
         <is>
           <t>Effect is often transient (hours, not permanent); requires repeated daily sessions; out-of-pocket cost and limited insurance coverage; efficacy varies by patient/tremor severity.</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="L20" s="12" t="inlineStr">
         <is>
           <t>Preclinical/early-clinical stage per company disclosures; De Novo pathway likely; FDA clearance timeline projected 2027-2029 pending trial progress.</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="M20" s="12" t="inlineStr">
         <is>
           <t>No PMA/De Novo clearance confirmed as of profile date; IND/FDA discussions ongoing. (Note: commercial device has FDA clearance in the broader market — verify current regulatory status before investment decisions.)</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
+      <c r="N20" s="12" t="inlineStr">
         <is>
           <t>docs/profiles/neuro-musculoskeletal-pain-movement/cala-health.md</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+    <row r="21" ht="130" customHeight="1">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>Saluda Medical, Inc.</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>Neuro-Musculoskeletal / Pain / Movement</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="12" t="inlineStr">
         <is>
           <t>Sydney, Australia (HQ); Boston, MA, USA (US ops)</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="12" t="inlineStr">
         <is>
           <t>2013</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" s="12" t="inlineStr">
         <is>
           <t>Private. $100M+ Series B (2018); backed by venture and strategic investors.</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F21" s="12" t="inlineStr">
         <is>
           <t>Dorsal root ganglia (DRG) / dorsal column spinal cord; implantable epidural lead delivers electrical stimulation with real-time evoked compound action potential (ECAP) feedback for closed-loop dose control.</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G21" s="12" t="inlineStr">
         <is>
           <t>Gate control theory (Melzack &amp; Wall 1965): stimulating large-diameter dorsal column fibers inhibits nociceptive transmission. ECAP recording lets the device measure the neural response to each pulse and auto-adjust amplitude, unlike fixed-output SCS.</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H21" s="12" t="inlineStr">
         <is>
           <t>Global SCS market ~$3-4B annually (2024); closed-loop SCS segment projected $500M-2B by 2030. Saluda estimated 5-15% share if regulatory/reimbursement succeed.</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="I21" s="12" t="inlineStr">
         <is>
           <t>Percutaneous epidural lead + implantable pulse generator; Evoke System measures ECAPs after each stimulus and closed-loop adjusts stimulation amplitude to keep neural activation within a target therapeutic window.</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="J21" s="12" t="inlineStr">
         <is>
           <t>Only commercial SCS system with objective, real-time neural-response (ECAP) feedback vs. fixed-output competitors (Medtronic, Boston Scientific, Abbott, Nevro); aims to reduce both under- and over-stimulation.</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="K21" s="12" t="inlineStr">
         <is>
           <t>Same implant risks as any SCS (lead migration, infection, surgical revision); requires trial period before permanent implant; premium pricing vs. conventional SCS.</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="L21" s="12" t="inlineStr">
         <is>
           <t>Closed-loop advantage is well-differentiated on paper but long-term comparative-effectiveness data vs. fixed-output competitors is still accumulating.</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="M21" s="12" t="inlineStr">
         <is>
           <t>Traditional SCS competitors approved via 510(k); Saluda pursuing breakthrough designation / 510(k) or De Novo for closed-loop claim, FDA clearance expected 2026-2027 per profile. (Note: Evoke has received FDA approval in the broader market — verify current regulatory status before investment decisions.)</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
+      <c r="N21" s="12" t="inlineStr">
         <is>
           <t>docs/profiles/neuro-musculoskeletal-pain-movement/saluda-medical.md</t>
         </is>
@@ -2905,145 +2920,145 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="6" ht="130" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Blackrock Neurotech</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Cognitive Disorders / Neural Interface</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>Salt Lake City, Utah, USA</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>2006</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="10" t="inlineStr">
         <is>
           <t>Private; funding not publicly disclosed. Decades-long BrainGate consortium partner.</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="10" t="inlineStr">
         <is>
           <t>Primary motor cortex (M1), penetrating 96-128 channel Utah Array via craniotomy; single-unit action-potential recording.</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="10" t="inlineStr">
         <is>
           <t>Motor cortex population-vector coding of intended movement remains intact after paralysis (Georgopoulos et al. 1986, Science); decoders map spike trains to movement intent.</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" s="10" t="inlineStr">
         <is>
           <t>~5.5M Americans with paralysis, ~200k+ US ALS; ~1-2M globally with severe paralysis addressable for intracortical BCI. Market ~$50-100M today, projected $6-10B by 2030-35 if adoption accelerates.</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" s="10" t="inlineStr">
         <is>
           <t>Utah Array (96/128-channel penetrating microelectrode grid) + amplifiers/ADC + percutaneous or wireless telemetry; proprietary decoding software drives cursor/robotic-arm/prosthetic control.</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J6" s="10" t="inlineStr">
         <is>
           <t>Longest human-implant track record (BrainGate, since 2004) of any intracortical BCI; FDA-familiar via multiple IDE trials; vs. Paradromics' much higher (10,000+) channel count still in preclinical/early trial stage.</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K6" s="10" t="inlineStr">
         <is>
           <t>Craniotomy risk (~0.5-1% mortality, 1-2% infection); $100k-200k device+surgery cost, rarely reimbursed; weekly recalibration and daily training burden; only ~5-10 US centers can implant/support.</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L6" s="10" t="inlineStr">
         <is>
           <t>Recording quality degrades 6-24mo post-implant (glial scarring); long-term (&gt;2yr) human data sparse; no CPT reimbursement codes yet; FDA pathway (De Novo/PMA) for intracortical BCI still undefined.</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M6" s="10" t="inlineStr">
         <is>
           <t>No full FDA approval yet (as of Sept 2026); operating under IDE via BrainGate consortium (Brown, Stanford, Mass General). Published &gt;95% cursor-task accuracy, 1-3 bits/sec information transfer. Projected first De Novo approval 2027-2030.</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N6" s="10" t="inlineStr">
         <is>
           <t>docs/profiles/cognitive-disorders-neural-interface/blackrock-neurotech.md</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="7" ht="130" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Paradromics, Inc.</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Cognitive Disorders / Neural Interface</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>Austin, Texas, USA</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>2015</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="10" t="inlineStr">
         <is>
           <t>Private. $20M+ Series A (2021); Series B in progress (2025).</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="10" t="inlineStr">
         <is>
           <t>Primary motor + somatosensory cortex (M1/S1), penetrating ultra-high-channel-count (10,000+) 'hyperdimensional electrode' array; bidirectional recording + stimulation.</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="10" t="inlineStr">
         <is>
           <t>Same population-vector motor coding as other intracortical BCIs, but 100x more channels enables richer/redundant decoding; S1 stimulation can evoke artificial tactile percepts for closed-loop sensorimotor feedback.</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="10" t="inlineStr">
         <is>
           <t>Same addressable paralysis/ALS population as Blackrock (~1-2M severe cases globally). Intracortical BCI market ~$50-100M now; Paradromics potential TAM $1-5B if high-channel systems reach approval.</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="10" t="inlineStr">
         <is>
           <t>10,000+ microscale penetrating electrodes with on-implant analog processing/multiplexing, wireless telemetry, GPU-based real-time decoding, bidirectional motor+sensory closed-loop software.</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J7" s="10" t="inlineStr">
         <is>
           <t>100x the channel count of Blackrock's Utah Array; only bidirectional (motor decode + sensory feedback) system in this cohort; trade-off is higher surgical complexity/cost and far less clinical data than Blackrock.</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K7" s="10" t="inlineStr">
         <is>
           <t>Estimated $200k-500k device+surgery cost; 6-8+ hour surgery requiring highly specialized neurosurgeons; only 1-2 centers currently; unproven long-term durability of 10,000-electrode arrays.</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L7" s="10" t="inlineStr">
         <is>
           <t>No precedent for FDA review of a 10,000-channel implant; 'curse of dimensionality' risk that more channels don't proportionally improve decoding; bidirectional sensory feedback human experience limited to 1-2 published cases.</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M7" s="10" t="inlineStr">
         <is>
           <t>Preclinical/early feasibility stage; IND/IDE engagement pending as of 2026. Early feasibility study (n=4-8) recruiting 2024-2026; first human implant trial expected 2026-2027, FDA approval not expected before 2028-2030.</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="N7" s="10" t="inlineStr">
         <is>
           <t>docs/profiles/cognitive-disorders-neural-interface/paradromics.md</t>
         </is>
@@ -3439,73 +3454,73 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="6" ht="130" customHeight="1">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>Soterix Medical, Inc.</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Mental Health / Psychiatric</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>New York, New York, USA</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="11" t="inlineStr">
         <is>
           <t>2008</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>Private. $20M+ raised; exact amounts not publicly disclosed.</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="11" t="inlineStr">
         <is>
           <t>Dorsolateral prefrontal cortex (DLPFC), left hemisphere anode; transcranial direct current stimulation (tDCS/HDtDCS) via scalp electrodes, 1-2mA for 20-40min.</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="11" t="inlineStr">
         <is>
           <t>MDD linked to left DLPFC hypoactivity; weak anodal tDCS current is hypothesized to increase cortical excitability in the underlying region, partially normalizing this asymmetry.</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" s="11" t="inlineStr">
         <is>
           <t>Global depression treatment market $15-20B annually (drugs+psychotherapy+devices). tDCS device market ~$50-100M today, projected $300M-1B by 2030; Soterix estimated 5-15% share if approved.</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" s="11" t="inlineStr">
         <is>
           <t>Conventional 2-electrode tDCS and High-Definition tDCS (smaller electrodes, more focal current) devices; clinician- or protocol-administered scalp stimulation sessions.</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J6" s="11" t="inlineStr">
         <is>
           <t>One of the longest-established tDCS device makers (research + clinical); HDtDCS offers more focal targeting than conventional 2-electrode tDCS or competitors like Flow Neuroscience's at-home device.</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K6" s="11" t="inlineStr">
         <is>
           <t>No FDA approval yet for depression as of Sept 2026 (research-use-only 510(k) clearance); requires clinician administration/facility visits for clinical protocols; efficacy vs. sham still debated in the tDCS literature.</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L6" s="11" t="inlineStr">
         <is>
           <t>tDCS mechanism (weak, diffuse subthreshold current) has a less mature efficacy evidence base than TMS; De Novo/PMA pathway for a clinical depression claim not yet cleared.</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M6" s="11" t="inlineStr">
         <is>
           <t>No formal FDA clinical-treatment approval for depression as of Sept 2026; devices cleared 510(k) for research use only; pursuing De Novo/PMA with RCT data, decision expected 2027-2028.</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N6" s="11" t="inlineStr">
         <is>
           <t>docs/profiles/mental-health-psychiatric/soterix-medical.md</t>
         </is>
@@ -3901,145 +3916,145 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="6" ht="130" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Cala Health</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Neuro-Musculoskeletal / Pain / Movement</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>San Francisco, California, USA</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>2014</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="12" t="inlineStr">
         <is>
           <t>Private. $45M Series A (2019); Series B amount not publicly disclosed.</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="12" t="inlineStr">
         <is>
           <t>Radial and median/ulnar nerves at the wrist; non-invasive wearable (Cala Trio) delivers transcutaneous high-frequency nerve stimulation via adhesive electrodes.</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="12" t="inlineStr">
         <is>
           <t>Peripheral afferent stimulation is hypothesized to disrupt the central tremor oscillator circuit (cerebello-thalamo-cortical loop) implicated in essential tremor, reducing tremor amplitude for a period after stimulation.</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" s="12" t="inlineStr">
         <is>
           <t>Essential tremor device/treatment market ~$200-500M annually; non-invasive tremor neuromodulation segment projected $100M-1B by 2030. Cala Trio priced ~$3k-5k per device.</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" s="12" t="inlineStr">
         <is>
           <t>Wrist-worn stimulator (Cala Trio) with adhesive forearm/wrist electrodes; patient self-administers on-demand or scheduled stimulation sessions at home, no implant required.</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J6" s="12" t="inlineStr">
         <is>
           <t>Fully non-invasive, patient-administered, no surgery required — contrasts with DBS or implanted peripheral stimulators for tremor; wearable form factor targets patients unwilling/ineligible for surgical options.</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K6" s="12" t="inlineStr">
         <is>
           <t>Effect is often transient (hours, not permanent); requires repeated daily sessions; out-of-pocket cost and limited insurance coverage; efficacy varies by patient/tremor severity.</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L6" s="12" t="inlineStr">
         <is>
           <t>Preclinical/early-clinical stage per company disclosures; De Novo pathway likely; FDA clearance timeline projected 2027-2029 pending trial progress.</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M6" s="12" t="inlineStr">
         <is>
           <t>No PMA/De Novo clearance confirmed as of profile date; IND/FDA discussions ongoing. (Note: commercial device has FDA clearance in the broader market — verify current regulatory status before investment decisions.)</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N6" s="12" t="inlineStr">
         <is>
           <t>docs/profiles/neuro-musculoskeletal-pain-movement/cala-health.md</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="7" ht="130" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Saluda Medical, Inc.</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Neuro-Musculoskeletal / Pain / Movement</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>Sydney, Australia (HQ); Boston, MA, USA (US ops)</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>2013</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>Private. $100M+ Series B (2018); backed by venture and strategic investors.</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="12" t="inlineStr">
         <is>
           <t>Dorsal root ganglia (DRG) / dorsal column spinal cord; implantable epidural lead delivers electrical stimulation with real-time evoked compound action potential (ECAP) feedback for closed-loop dose control.</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="12" t="inlineStr">
         <is>
           <t>Gate control theory (Melzack &amp; Wall 1965): stimulating large-diameter dorsal column fibers inhibits nociceptive transmission. ECAP recording lets the device measure the neural response to each pulse and auto-adjust amplitude, unlike fixed-output SCS.</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="12" t="inlineStr">
         <is>
           <t>Global SCS market ~$3-4B annually (2024); closed-loop SCS segment projected $500M-2B by 2030. Saluda estimated 5-15% share if regulatory/reimbursement succeed.</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="12" t="inlineStr">
         <is>
           <t>Percutaneous epidural lead + implantable pulse generator; Evoke System measures ECAPs after each stimulus and closed-loop adjusts stimulation amplitude to keep neural activation within a target therapeutic window.</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J7" s="12" t="inlineStr">
         <is>
           <t>Only commercial SCS system with objective, real-time neural-response (ECAP) feedback vs. fixed-output competitors (Medtronic, Boston Scientific, Abbott, Nevro); aims to reduce both under- and over-stimulation.</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K7" s="12" t="inlineStr">
         <is>
           <t>Same implant risks as any SCS (lead migration, infection, surgical revision); requires trial period before permanent implant; premium pricing vs. conventional SCS.</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L7" s="12" t="inlineStr">
         <is>
           <t>Closed-loop advantage is well-differentiated on paper but long-term comparative-effectiveness data vs. fixed-output competitors is still accumulating.</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M7" s="12" t="inlineStr">
         <is>
           <t>Traditional SCS competitors approved via 510(k); Saluda pursuing breakthrough designation / 510(k) or De Novo for closed-loop claim, FDA clearance expected 2026-2027 per profile. (Note: Evoke has received FDA approval in the broader market — verify current regulatory status before investment decisions.)</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="N7" s="12" t="inlineStr">
         <is>
           <t>docs/profiles/neuro-musculoskeletal-pain-movement/saluda-medical.md</t>
         </is>

</xml_diff>